<commit_message>
🚀 Sistema de Gestión de Stock - Versión Completa y Optimizada
</commit_message>
<xml_diff>
--- a/data_sources/catalogs/codigos_especiales.xlsx
+++ b/data_sources/catalogs/codigos_especiales.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ccusi\Documents\Proyect_Coder\gestion_de_stock\datos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ccusi\Documents\Proyect_Coder\gestion_de_stock\data_sources\catalogs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C733AE04-6F1C-458E-8D4D-85905D58F542}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43BECA69-0BDA-4F12-8DA5-D8A820BF1F48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="510" yWindow="600" windowWidth="18000" windowHeight="11010" xr2:uid="{325F3910-60B6-4BEE-B8EF-465835BC1720}"/>
+    <workbookView xWindow="315" yWindow="3615" windowWidth="21600" windowHeight="11385" xr2:uid="{325F3910-60B6-4BEE-B8EF-465835BC1720}"/>
   </bookViews>
   <sheets>
     <sheet name="especiales" sheetId="1" r:id="rId1"/>
@@ -34,15 +34,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="32">
   <si>
     <t>codigo</t>
   </si>
   <si>
     <t>orden</t>
-  </si>
-  <si>
-    <t>u_por_caja</t>
   </si>
   <si>
     <t>motivo</t>
@@ -196,9 +193,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
@@ -482,336 +478,324 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E015A6FE-854C-4D0C-BFD8-8D173EA7CD2D}">
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="C2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2" s="1">
-        <v>60</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="C4" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="2"/>
-      <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="C3" s="1">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
         <v>5</v>
       </c>
-      <c r="B4">
-        <v>3</v>
-      </c>
-      <c r="C4" s="1">
-        <v>60</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="C5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7">
         <v>6</v>
       </c>
-      <c r="B5">
-        <v>4</v>
-      </c>
-      <c r="D5" t="s">
+      <c r="B7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8">
         <v>7</v>
       </c>
-      <c r="B6">
-        <v>5</v>
-      </c>
-      <c r="D6" t="s">
+      <c r="B8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>11</v>
+      </c>
+      <c r="C14" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7">
-        <v>6</v>
-      </c>
-      <c r="D7" t="s">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8">
-        <v>7</v>
-      </c>
-      <c r="D8" t="s">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>12</v>
+      </c>
+      <c r="C16" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>14</v>
+      </c>
+      <c r="C17" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>15</v>
+      </c>
+      <c r="C19" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>16</v>
+      </c>
+      <c r="C20" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
         <v>10</v>
       </c>
-      <c r="B9">
-        <v>8</v>
-      </c>
-      <c r="D9" t="s">
+      <c r="C22" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C23" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="s">
+        <v>18</v>
+      </c>
+      <c r="C24" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>19</v>
+      </c>
+      <c r="C26" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>20</v>
+      </c>
+      <c r="C27" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28">
         <v>27</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>11</v>
-      </c>
-      <c r="B10">
-        <v>9</v>
-      </c>
-      <c r="D10" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B11">
+      <c r="B28" t="s">
         <v>10</v>
       </c>
-      <c r="D11" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12">
-        <v>11</v>
-      </c>
-      <c r="D12" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B13">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>12</v>
-      </c>
-      <c r="B14">
-        <v>13</v>
-      </c>
-      <c r="D14" t="s">
+      <c r="C28" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29">
         <v>28</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>14</v>
-      </c>
-      <c r="B15">
-        <v>14</v>
-      </c>
-      <c r="D15" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>13</v>
-      </c>
-      <c r="B16">
-        <v>15</v>
-      </c>
-      <c r="D16" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>15</v>
-      </c>
-      <c r="B17">
-        <v>16</v>
-      </c>
-      <c r="D17" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B18">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>16</v>
-      </c>
-      <c r="B19">
-        <v>18</v>
-      </c>
-      <c r="D19" t="s">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30">
         <v>29</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>17</v>
-      </c>
-      <c r="B20">
-        <v>19</v>
-      </c>
-      <c r="D20" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B21">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>11</v>
-      </c>
-      <c r="B22">
+      <c r="B30" t="s">
         <v>21</v>
       </c>
-      <c r="D22" t="s">
+      <c r="C30" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31">
         <v>30</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>18</v>
-      </c>
-      <c r="B23">
+      <c r="B31" t="s">
         <v>22</v>
       </c>
-      <c r="D23" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>19</v>
-      </c>
-      <c r="B24">
+      <c r="C31" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="s">
         <v>23</v>
       </c>
-      <c r="D24" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B25">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B26">
-        <v>25</v>
-      </c>
-      <c r="D26" t="s">
+      <c r="C32" t="s">
         <v>31</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>21</v>
-      </c>
-      <c r="B27">
-        <v>26</v>
-      </c>
-      <c r="D27" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>11</v>
-      </c>
-      <c r="B28">
-        <v>27</v>
-      </c>
-      <c r="D28" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B29">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>22</v>
-      </c>
-      <c r="B30">
-        <v>29</v>
-      </c>
-      <c r="D30" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>23</v>
-      </c>
-      <c r="B31">
-        <v>30</v>
-      </c>
-      <c r="D31" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>24</v>
-      </c>
-      <c r="B32">
-        <v>31</v>
-      </c>
-      <c r="D32" t="s">
-        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>